<commit_message>
Link penalty records to FIA decision documents
Add a Doc column with a PDF link to the raw data, race log, driver,
team, race and steward tables, include Doc_URL in the CSV export, and
fill Doc_URL for 2026 Madrid, Azerbaijan and Singapore.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P140"/>
+  <dimension ref="A1:Q140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.109375" customWidth="1" min="2" max="2"/>
@@ -462,6 +462,7 @@
     <col width="15.44140625" customWidth="1" min="10" max="10"/>
     <col width="7.88671875" customWidth="1" min="15" max="15"/>
     <col width="33" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,6 +544,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Stewards</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_URL</t>
         </is>
       </c>
     </row>
@@ -7485,12 +7491,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P164"/>
+  <dimension ref="A1:Q164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6.109375" customWidth="1" min="6" max="6"/>
     <col width="22.5546875" customWidth="1" min="7" max="7"/>
     <col width="13.77734375" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7572,6 +7579,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Stewards</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_URL</t>
         </is>
       </c>
     </row>
@@ -16023,11 +16035,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P216"/>
+  <dimension ref="A1:Q216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="26.88671875" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16109,6 +16122,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Stewards</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_URL</t>
         </is>
       </c>
     </row>
@@ -27247,11 +27265,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P228"/>
+  <dimension ref="A1:Q228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18.109375" customWidth="1" min="7" max="7"/>
     <col width="13.44140625" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -27333,6 +27352,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Stewards</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_URL</t>
         </is>
       </c>
     </row>
@@ -39080,7 +39104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P245"/>
+  <dimension ref="A1:Q245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.77734375" customWidth="1" min="6" max="6"/>
@@ -39088,6 +39112,7 @@
     <col width="31.6640625" customWidth="1" min="8" max="8"/>
     <col width="13.6640625" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -39169,6 +39194,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Stewards</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_URL</t>
         </is>
       </c>
     </row>
@@ -51952,12 +51982,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P254"/>
+  <dimension ref="A1:Q254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="42.5546875" customWidth="1" min="7" max="7"/>
     <col width="25.21875" customWidth="1" min="8" max="8"/>
     <col width="25.88671875" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -52039,6 +52070,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Stewards</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_URL</t>
         </is>
       </c>
     </row>
@@ -65013,7 +65049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P253"/>
+  <dimension ref="A1:Q253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="32.21875" customWidth="1" min="7" max="7"/>
@@ -65023,6 +65059,7 @@
     <col width="12.21875" customWidth="1" min="13" max="13"/>
     <col width="6.109375" customWidth="1" min="14" max="14"/>
     <col width="26.109375" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -65106,6 +65143,11 @@
           <t>Stewards</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -75061,6 +75103,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_11_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -75112,6 +75159,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_11_-_second_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -75165,6 +75217,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_23_-_leaving_the_track_and_re-joining_unsafely_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -75213,6 +75270,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_77_-_failure_to_follow_race_directors_instructions_escape_roads.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -75259,6 +75321,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_1_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -75305,6 +75372,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_18_-_pu_elements_changed.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -75356,6 +75428,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_55_-_impeding_of_car_77.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -75404,6 +75481,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_5_-_failure_to_follow_rd_instructions_scl2_-_scl1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -75452,6 +75534,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_12_-_failure_to_follow_rd_instructions_scl2_-_scl1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -75500,6 +75587,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_63_-_failure_to_follow_race_director_instructions_-_scl2_-_scl1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -75553,6 +75645,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_16_-_failure_to_follow_rd_instructions_scl2_-_scl1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -75604,6 +75701,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_22_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -75660,6 +75762,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_55_-_causing_a_collision_with_car_14.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -75706,6 +75813,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_10_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -75764,6 +75876,11 @@
           <t>Felix Holter, Natalie Corsmit, Mathieu Remmerie, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_spanish_grand_prix_-_infringement_-_car_5_-_moving_under_braking.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -75822,6 +75939,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_77_-_overtaking_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -75868,6 +75990,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_18_-_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -75914,6 +76041,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_14_-_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -75967,6 +76099,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_44_-_impeding_car_30.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -76013,6 +76150,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_14_-_pu_element.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -76066,6 +76208,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_55_-_failure_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -76119,6 +76266,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_41_-_leaving_the_track_in_turn_15.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -76170,6 +76322,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_11_-_impeding_car_81.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -76229,6 +76386,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_55_-_failure_to_slow_for_yellow_flags_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -76285,6 +76447,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_43_-_collision_with_car_10_in_turn_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -76338,6 +76505,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_decision_-_car_41_-_collision_with_car_30_in_turn_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -76399,6 +76571,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_5_-_overtaking_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -76447,6 +76624,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_decision_-_car_77_-_turn_15_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -76500,6 +76682,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_6_-_failing_to_follow_race_directors_instructions_-_practice_start.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -76553,6 +76740,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Khatuna Julakidze, Derek Warwick, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_azerbaijan_grand_prix_-_infringement_-_car_55_-_failing_to_follow_race_directors_instructions_-_practice_start.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -76599,6 +76791,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_63_-_changes_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -76657,6 +76854,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_55_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -76715,6 +76917,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_3_-_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -76768,6 +76975,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_11_-_causing_a_collision_with_car_18.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -76816,6 +77028,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_18_-_alleged_causing_a_collision_with_car_11.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -76864,6 +77081,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_41_-_alleged_driving_opposite_direction.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -76917,6 +77139,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_23_-_causing_a_collision_with_car_5.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -76970,6 +77197,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_77_-_causing_a_collision_with_car_23.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -77018,6 +77250,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_81_-_alleged_causing_a_collision_with_car_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -77066,6 +77303,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_1_-_alleged_causing_a_collision_with_car_81.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -77119,6 +77361,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_87_-_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -77165,6 +77412,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_63_-_additional_changes_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -77218,6 +77470,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_6_-_pu_elements_and_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -77271,6 +77528,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_18_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -77324,6 +77586,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_14_-_pu_element_and_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -77377,6 +77644,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_27_-_impeding_of_car_55.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -77430,6 +77702,11 @@
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_18_-_failure_to_follow_race_directors_instructions_-_practice_start.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -77481,6 +77758,11 @@
       <c r="P253" t="inlineStr">
         <is>
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_44_-_alleged_leaving_the_track_and_gaining_an_advantage.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FIA document links for 2026 Australia, Spain, Austria, Great Britain and Belgium
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="3" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2020" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2021" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2022" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2023" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2020" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2021" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2022" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2023" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2024" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65196,6 +65196,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_infringement_-_car_63_-_failure_to_follow_race_director_instruction_-_practice_start.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -65249,6 +65254,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_infringement_-_car_63_-_pit_lane_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -65302,6 +65312,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_decision_-_car_43_-_allegedly_driving_unnecessarily_slow.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -65353,6 +65368,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_infringement_-_car_12_-_released_in_an_unsafe_condition.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -65404,6 +65424,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_infringement_-_car_10_-_released_in_an_unsafe_condition.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -65457,6 +65482,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_decision_-_car_12_-_alleged_pitlane_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -65505,6 +65535,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_decision_-_car_27_-_start_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -65553,6 +65588,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_infringement_-_car_43_-_grid_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -65606,6 +65646,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_decision_-_car_31_-_alleged_causing_a_collision_with_car_10.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -65659,6 +65704,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_decision_-_car_10_-_alleged_causing_a_collision_with_car_31.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -65702,6 +65752,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_decision_-_car_31_-_allegedly_driving_unnecessarily_slowly.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -65750,6 +65805,11 @@
           <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_australian_grand_prix_-_decision_-_car_11_-_alleged_forcing_another_driver_off_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -70156,6 +70216,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_14_-_pit_exit_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -70202,6 +70267,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_77_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -70248,6 +70318,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_11_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -70294,6 +70369,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_18_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -70342,6 +70422,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_12_-_driving_erratically.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -70390,6 +70475,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_16_-_impeding_of_car_27.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -70438,6 +70528,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_14_-_pu_elements_and_changes_used_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -70481,6 +70576,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_decision_-_car_27_-_alleged_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -70524,6 +70624,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_decision_-_car_41_-_alleged_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -70573,6 +70678,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_43_-_failing_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -70624,6 +70734,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_23_-_start_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -70675,6 +70790,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_55_-_start_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -70721,6 +70841,11 @@
           <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
         </is>
       </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_barcelona-catalunya_grand_prix_-_infringement_-_car_12_-_leaving_the_track_without_a_justifiable_reason_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -70767,6 +70892,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_infringement_-_car_14_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -70810,6 +70940,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_infringement_-_car_6_-_failing_to_follow_race_directors_instructions_sc2-sc1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -70858,6 +70993,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_decision_-_car_81_-_alleged_failing_to_follow_race_directors_instructions_sc2-sc1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -70901,6 +71041,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_decision_-_car_30_-_failure_to_follow_race_directors_instructions_-_practice_starts.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -70944,6 +71089,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_decision_-_car_23_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -70987,6 +71137,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_decision_-_car_18_-_alleged_ignoring_blue_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -71030,6 +71185,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_decision_-_car_14_-_alleged_ignoring_blue_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -71073,6 +71233,11 @@
           <t>Felix Holter, Loic Bacquelaine, Pedro Lamy, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_austrian_grand_prix_-_decision_-_car_11_-_alleged_false_start_-_moving_before_signal.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -71174,6 +71339,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_55_-_overtaking_the_safety_car.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -71222,6 +71392,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_44_-_yellow_flags_-_failing_to_slow.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -71268,6 +71443,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_44_-_false_start_-_moving_before_start_signal.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -71314,6 +71494,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_41_-_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -71613,6 +71798,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_23_-_causing_a_collision_with_car_87.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -71659,6 +71849,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_18_-_pu_elements_changed.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -71705,6 +71900,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_18_-_leaving_the_track_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -71751,6 +71951,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_18_-_leaving_the_track_multiple_times_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -71797,6 +72002,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_18_-_leaving_the_track_multiple_times_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -71843,6 +72053,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_12_-_leaving_the_track_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -71945,6 +72160,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_10_-_impeding_of_car_18.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -72034,6 +72254,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_55_-_change_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -72087,6 +72312,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_55_-_crossing_the_white_line_at_pit_entry.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -72143,6 +72373,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_31_-_media_commitment.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -72194,6 +72429,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_44_-_causing_a_collision_with_car_63_in_turn_5.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -72240,6 +72480,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_34_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -72286,6 +72531,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_corrected_infringement_-_car_6_-_changes_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -72332,6 +72582,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_corrected_infringement_-_car_14_-_change_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -72380,6 +72635,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_decision_-_car_16_-_collision_with_car_81_in_turn_5.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -72428,6 +72688,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_decision_-_car_55_-_alleged_failure_to_slow_for_double_yellow_flags_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -72474,6 +72739,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_1_-_change_to_pu_element.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -72580,6 +72850,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_27_-_failure_to_slow_under_double_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -72631,6 +72906,11 @@
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_ferrari_-_car_16_return_of_tyres.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -72685,6 +72965,11 @@
       <c r="P156" t="inlineStr">
         <is>
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_ferrari_-_unsafe_release_of_car_44.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 2026 Bahrain GP in Malaysia as Malaysia* (Round 16)
Add the race's 11 stewards decisions with FIA document links, move
Singapore to Round 17, add the race to the 2026 calendar, and set
Albon's Belgium rear-lights row to Pre-Race with its document link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -65049,7 +65049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q253"/>
+  <dimension ref="A1:Q264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="32.21875" customWidth="1" min="7" max="7"/>
@@ -72769,7 +72769,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Pre-Race</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -72795,6 +72795,11 @@
       <c r="P153" t="inlineStr">
         <is>
           <t>Gerd Ennser, Matthew Selley, Alfonso Orihuela, Pedro Lamy, Loic Bacquelaine</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_belgian_grand_prix_-_infringement_-_car_23_-_car_safety_lights_.pdf</t>
         </is>
       </c>
     </row>
@@ -77040,22 +77045,22 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>George Russell</t>
+          <t>Isack Hadjar</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Mercedes</t>
+          <t>Red Bull</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>FP1</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -77069,16 +77074,16 @@
         </is>
       </c>
       <c r="M236" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q236" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_63_-_changes_to_pu_elements.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_6_-_changes_to_pu_elements.pdf</t>
         </is>
       </c>
     </row>
@@ -77091,32 +77096,27 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Carlos Sainz</t>
+          <t>Franco Colapinto</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Williams</t>
+          <t>Alpine</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>SQ</t>
+          <t>FP1</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Changes made under parc ferme</t>
-        </is>
-      </c>
-      <c r="H237" t="inlineStr">
-        <is>
-          <t>Suspension setup changed under parc ferme</t>
+          <t>New power unit element(s)</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
@@ -77124,24 +77124,17 @@
           <t>Grid Penalty</t>
         </is>
       </c>
-      <c r="M237" t="inlineStr">
-        <is>
-          <t>Pit Lane</t>
-        </is>
-      </c>
-      <c r="O237" t="inlineStr">
-        <is>
-          <t>Started the Sprint from the pit lane</t>
-        </is>
+      <c r="M237" t="n">
+        <v>10</v>
       </c>
       <c r="P237" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q237" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_55_-_changes_made_during_parc_ferme.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_43_-_changes_to_pu_elements.pdf</t>
         </is>
       </c>
     </row>
@@ -77154,57 +77147,45 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Max Verstappen</t>
+          <t>Arvid Lindblad</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Red Bull</t>
+          <t>Racing Bulls</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>SQ</t>
+          <t>FP1</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Yellow Flag Infringement</t>
-        </is>
-      </c>
-      <c r="H238" t="inlineStr">
-        <is>
-          <t>Overtook under single yellow</t>
-        </is>
-      </c>
-      <c r="I238" t="inlineStr">
-        <is>
-          <t>Lewis Hamilton</t>
+          <t>New power unit element(s)</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>No Further Action</t>
-        </is>
-      </c>
-      <c r="O238" t="inlineStr">
-        <is>
-          <t>Breach confirmed but no penalty, driver lifted and closing speed was too high to avoid the overtake</t>
-        </is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M238" t="n">
+        <v>30</v>
       </c>
       <c r="P238" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q238" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_3_-_yellow_flag_infringement.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_41_-_changes_to_pu_elements.pdf</t>
         </is>
       </c>
     </row>
@@ -77217,52 +77198,55 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Sergio Perez</t>
+          <t>Lewis Hamilton</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Cadillac</t>
+          <t>Ferrari</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>FP2</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Causing a Collision</t>
+          <t>Impeding</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>Lance Stroll</t>
+          <t>Gabriel Bortoleto</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>No Further Action</t>
-        </is>
+          <t>Warning, Fine</t>
+        </is>
+      </c>
+      <c r="L239" t="n">
+        <v>10000</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>Predominantly to blame. Stewards would have given a 5 second time penalty, but the driver was not classified and 5 second penalties are not converted to grid drops</t>
+          <t>Team fined for not warning the driver, whose right mirror was damaged</t>
         </is>
       </c>
       <c r="P239" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q239" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_11_-_causing_a_collision_with_car_18.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_44_-_impeding_of_car_5.pdf</t>
         </is>
       </c>
     </row>
@@ -77275,7 +77259,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -77290,32 +77274,32 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>Causing a Collision</t>
-        </is>
-      </c>
-      <c r="I240" t="inlineStr">
-        <is>
-          <t>Sergio Perez</t>
+          <t>Failure to follow race director's instructions</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Exceeded time limit between the safety car lines</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>No Further Action</t>
+          <t>Warning</t>
         </is>
       </c>
       <c r="P240" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q240" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_18_-_alleged_causing_a_collision_with_car_11.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_18_-_failure_to_follow_race_directors_instructions_sc2-sc1_time_1st_offence.pdf</t>
         </is>
       </c>
     </row>
@@ -77328,47 +77312,52 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Arvid Lindblad</t>
+          <t>Lance Stroll</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Racing Bulls</t>
+          <t>Aston Martin</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>Unsafe Act</t>
+          <t>Failure to follow race director's instructions</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>Drove in the wrong direction at Turn 5 after a spin</t>
+          <t>Exceeded time limit between the safety car lines</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>No Further Action</t>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>Second breach in the same session</t>
         </is>
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q241" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_41_-_alleged_driving_opposite_direction.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_18_-_failure_to_follow_race_directors_instructions_sc2-sc1_time_2nd_offence.pdf</t>
         </is>
       </c>
     </row>
@@ -77381,12 +77370,12 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Alexander Albon</t>
+          <t>Carlos Sainz</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -77396,37 +77385,35 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Pre-Race</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>Causing a Collision</t>
-        </is>
-      </c>
-      <c r="I242" t="inlineStr">
-        <is>
-          <t>Gabriel Bortoleto</t>
+          <t>Pit Lane Speeding</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>No Further Action</t>
-        </is>
+          <t>Fine</t>
+        </is>
+      </c>
+      <c r="L242" t="n">
+        <v>100</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>Stewards would have given a 5 second time penalty, but the driver retired and 5 second penalties are not converted to grid drops</t>
+          <t>Recon. Laps. 80.3 km/h</t>
         </is>
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q242" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_23_-_causing_a_collision_with_car_5.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_55_-_pit_lane_speeding.pdf</t>
         </is>
       </c>
     </row>
@@ -77439,22 +77426,22 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Valtteri Bottas</t>
+          <t>Gabriel Bortoleto</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Cadillac</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -77464,27 +77451,30 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>Alexander Albon</t>
+          <t>Carlos Sainz</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>No Further Action</t>
-        </is>
+          <t>Time Penalty</t>
+        </is>
+      </c>
+      <c r="K243" t="n">
+        <v>10</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>Stewards would have given a 5 second time penalty, but the driver retired and 5 second penalties are not converted to grid drops</t>
+          <t>Restart incident but first-lap leniency not applied</t>
         </is>
       </c>
       <c r="P243" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q243" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_77_-_causing_a_collision_with_car_23.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_5_-_causing_a_collision_with_car_55.pdf</t>
         </is>
       </c>
     </row>
@@ -77497,34 +77487,39 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
+          <t>Alexander Albon</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Driving Erratically</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>Slowed sharply approaching pit entry to meet the delta time</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
           <t>Oscar Piastri</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>McLaren</t>
-        </is>
-      </c>
-      <c r="F244" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="G244" t="inlineStr">
-        <is>
-          <t>Causing a Collision</t>
-        </is>
-      </c>
-      <c r="I244" t="inlineStr">
-        <is>
-          <t>Lando Norris</t>
-        </is>
-      </c>
       <c r="J244" t="inlineStr">
         <is>
           <t>No Further Action</t>
@@ -77532,12 +77527,12 @@
       </c>
       <c r="P244" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q244" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_81_-_alleged_causing_a_collision_with_car_1.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_decision_-_car_23_-_alleged_driving_erratically.pdf</t>
         </is>
       </c>
     </row>
@@ -77550,47 +77545,55 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Lando Norris</t>
+          <t>Nico Hulkenberg</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>McLaren</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>Causing a Collision</t>
-        </is>
-      </c>
-      <c r="I245" t="inlineStr">
-        <is>
-          <t>Oscar Piastri</t>
+          <t>Unsafe Release</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>Release light turned green while a mechanic was still in front of the car</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>No Further Action</t>
+          <t>Fine</t>
+        </is>
+      </c>
+      <c r="L245" t="n">
+        <v>30000</v>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>20000 of fine is suspended for the rest of the season. Stewards ruled no unsafe release, but the premature green light created an unsafe situation</t>
         </is>
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q245" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_1_-_alleged_causing_a_collision_with_car_81.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_27_-_unsafe_release.pdf</t>
         </is>
       </c>
     </row>
@@ -77603,52 +77606,57 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Malaysia*</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Oliver Bearman</t>
+          <t>Lando Norris</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Haas</t>
+          <t>McLaren</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>Failure to follow race director's instructions</t>
+          <t>Driving Erratically</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>Exceeded time limit between the safety car lines</t>
+          <t>Misjudged closing speed behind the Safety Car and avoided the cars ahead through the gravel</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Oscar Piastri</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>No Further Action</t>
+          <t>Reprimand</t>
         </is>
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>Slowed to let another car pass</t>
+          <t>Driver's first reprimand of the season</t>
         </is>
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+          <t>Gerd Ennser, Mathieu Remmerie, Pedro Lamy, Mazen Al Hilli</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_87_-_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_bahrain_grand_prix_in_malaysia_-_infringement_-_car_1_-_alleged_driving_erratically.pdf</t>
         </is>
       </c>
     </row>
@@ -77657,7 +77665,7 @@
         <v>2026</v>
       </c>
       <c r="B247" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -77676,7 +77684,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>R</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -77690,7 +77698,7 @@
         </is>
       </c>
       <c r="M247" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="P247" t="inlineStr">
         <is>
@@ -77699,7 +77707,7 @@
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_63_-_additional_changes_to_pu_elements.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_63_-_changes_to_pu_elements.pdf</t>
         </is>
       </c>
     </row>
@@ -77708,7 +77716,7 @@
         <v>2026</v>
       </c>
       <c r="B248" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
@@ -77717,17 +77725,17 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Isack Hadjar</t>
+          <t>Carlos Sainz</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Red Bull</t>
+          <t>Williams</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>SQ</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -77737,7 +77745,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>New PU elements fitted and suspension setup changed under parc ferme</t>
+          <t>Suspension setup changed under parc ferme</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -77750,6 +77758,11 @@
           <t>Pit Lane</t>
         </is>
       </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>Started the Sprint from the pit lane</t>
+        </is>
+      </c>
       <c r="P248" t="inlineStr">
         <is>
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
@@ -77757,7 +77770,7 @@
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_6_-_pu_elements_and_changes_made_during_parc_ferme.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_55_-_changes_made_during_parc_ferme.pdf</t>
         </is>
       </c>
     </row>
@@ -77766,7 +77779,7 @@
         <v>2026</v>
       </c>
       <c r="B249" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
@@ -77775,37 +77788,42 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Lance Stroll</t>
+          <t>Max Verstappen</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Aston Martin</t>
+          <t>Red Bull</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>SQ</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>Changes made under parc ferme</t>
+          <t>Yellow Flag Infringement</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>Suspension setup changed and work beyond covers-on time under parc ferme</t>
+          <t>Overtook under single yellow</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Lewis Hamilton</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>Grid Penalty</t>
-        </is>
-      </c>
-      <c r="M249" t="inlineStr">
-        <is>
-          <t>Pit Lane</t>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>Breach confirmed but no penalty, driver lifted and closing speed was too high to avoid the overtake</t>
         </is>
       </c>
       <c r="P249" t="inlineStr">
@@ -77815,7 +77833,7 @@
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_18_-_changes_made_during_parc_ferme.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_3_-_yellow_flag_infringement.pdf</t>
         </is>
       </c>
     </row>
@@ -77824,7 +77842,7 @@
         <v>2026</v>
       </c>
       <c r="B250" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -77833,37 +77851,37 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Fernando Alonso</t>
+          <t>Sergio Perez</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Aston Martin</t>
+          <t>Cadillac</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>Changes made under parc ferme</t>
-        </is>
-      </c>
-      <c r="H250" t="inlineStr">
-        <is>
-          <t>New PU element, suspension setup changed and work beyond covers-on time under parc ferme</t>
+          <t>Causing a Collision</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>Grid Penalty</t>
-        </is>
-      </c>
-      <c r="M250" t="inlineStr">
-        <is>
-          <t>Pit Lane</t>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>Predominantly to blame. Stewards would have given a 5 second time penalty, but the driver was not classified and 5 second penalties are not converted to grid drops</t>
         </is>
       </c>
       <c r="P250" t="inlineStr">
@@ -77873,7 +77891,7 @@
       </c>
       <c r="Q250" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_14_-_pu_element_and_changes_made_during_parc_ferme.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_11_-_causing_a_collision_with_car_18.pdf</t>
         </is>
       </c>
     </row>
@@ -77882,7 +77900,7 @@
         <v>2026</v>
       </c>
       <c r="B251" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
@@ -77891,27 +77909,27 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Nico Hulkenberg</t>
+          <t>Lance Stroll</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>Aston Martin</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>Impeding</t>
+          <t>Causing a Collision</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Carlos Sainz</t>
+          <t>Sergio Perez</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
@@ -77919,11 +77937,6 @@
           <t>No Further Action</t>
         </is>
       </c>
-      <c r="O251" t="inlineStr">
-        <is>
-          <t>Impeding confirmed but no penalty, team relied on official timing data that was briefly out of sync</t>
-        </is>
-      </c>
       <c r="P251" t="inlineStr">
         <is>
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
@@ -77931,7 +77944,7 @@
       </c>
       <c r="Q251" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_27_-_impeding_of_car_55.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_18_-_alleged_causing_a_collision_with_car_11.pdf</t>
         </is>
       </c>
     </row>
@@ -77940,7 +77953,7 @@
         <v>2026</v>
       </c>
       <c r="B252" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
@@ -77949,37 +77962,32 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Lance Stroll</t>
+          <t>Arvid Lindblad</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Aston Martin</t>
+          <t>Racing Bulls</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Pre-Race</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>Failure to follow race director's instructions</t>
+          <t>Unsafe Act</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>Did not cross the white line at pit exit when not performing a practice start</t>
+          <t>Drove in the wrong direction at Turn 5 after a spin</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="O252" t="inlineStr">
-        <is>
-          <t>Recon. Laps</t>
+          <t>No Further Action</t>
         </is>
       </c>
       <c r="P252" t="inlineStr">
@@ -77989,7 +77997,7 @@
       </c>
       <c r="Q252" t="inlineStr">
         <is>
-          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_18_-_failure_to_follow_race_directors_instructions_-_practice_start.pdf</t>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_41_-_alleged_driving_opposite_direction.pdf</t>
         </is>
       </c>
     </row>
@@ -77998,7 +78006,7 @@
         <v>2026</v>
       </c>
       <c r="B253" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
@@ -78007,45 +78015,666 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
+          <t>Alexander Albon</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Causing a Collision</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>Stewards would have given a 5 second time penalty, but the driver retired and 5 second penalties are not converted to grid drops</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_23_-_causing_a_collision_with_car_5.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B254" t="n">
+        <v>17</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Valtteri Bottas</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Causing a Collision</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Alexander Albon</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>Stewards would have given a 5 second time penalty, but the driver retired and 5 second penalties are not converted to grid drops</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_77_-_causing_a_collision_with_car_23.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B255" t="n">
+        <v>17</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Oscar Piastri</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Causing a Collision</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Lando Norris</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_81_-_alleged_causing_a_collision_with_car_1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B256" t="n">
+        <v>17</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Lando Norris</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>McLaren</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Causing a Collision</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Oscar Piastri</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_1_-_alleged_causing_a_collision_with_car_81.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B257" t="n">
+        <v>17</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Oliver Bearman</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Failure to follow race director's instructions</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Exceeded time limit between the safety car lines</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>Slowed to let another car pass</t>
+        </is>
+      </c>
+      <c r="P257" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_87_-_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B258" t="n">
+        <v>17</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>George Russell</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>New power unit element(s)</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M258" t="n">
+        <v>20</v>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_63_-_additional_changes_to_pu_elements.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B259" t="n">
+        <v>17</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Isack Hadjar</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Changes made under parc ferme</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>New PU elements fitted and suspension setup changed under parc ferme</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>Pit Lane</t>
+        </is>
+      </c>
+      <c r="P259" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_6_-_pu_elements_and_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B260" t="n">
+        <v>17</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Changes made under parc ferme</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Suspension setup changed and work beyond covers-on time under parc ferme</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>Pit Lane</t>
+        </is>
+      </c>
+      <c r="P260" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_18_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B261" t="n">
+        <v>17</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Fernando Alonso</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Changes made under parc ferme</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>New PU element, suspension setup changed and work beyond covers-on time under parc ferme</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>Pit Lane</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_14_-_pu_element_and_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B262" t="n">
+        <v>17</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Nico Hulkenberg</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Impeding</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Carlos Sainz</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>Impeding confirmed but no penalty, team relied on official timing data that was briefly out of sync</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_27_-_impeding_of_car_55.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B263" t="n">
+        <v>17</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Pre-Race</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Failure to follow race director's instructions</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Did not cross the white line at pit exit when not performing a practice start</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>Recon. Laps</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_infringement_-_car_18_-_failure_to_follow_race_directors_instructions_-_practice_start.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B264" t="n">
+        <v>17</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
           <t>Lewis Hamilton</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr">
+      <c r="E264" t="inlineStr">
         <is>
           <t>Ferrari</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr">
+      <c r="F264" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr">
+      <c r="G264" t="inlineStr">
         <is>
           <t>Leaving the Track and Gaining an Advantage</t>
         </is>
       </c>
-      <c r="I253" t="inlineStr">
+      <c r="I264" t="inlineStr">
         <is>
           <t>Lando Norris</t>
         </is>
       </c>
-      <c r="J253" t="inlineStr">
+      <c r="J264" t="inlineStr">
         <is>
           <t>No Further Action</t>
         </is>
       </c>
-      <c r="O253" t="inlineStr">
+      <c r="O264" t="inlineStr">
         <is>
           <t>Norris also left the track, both rejoined in the correct order</t>
         </is>
       </c>
-      <c r="P253" t="inlineStr">
+      <c r="P264" t="inlineStr">
         <is>
           <t>Felix Holter, Matthew Selley, Pedro Lamy, Paul Ng</t>
         </is>
       </c>
-      <c r="Q253" t="inlineStr">
+      <c r="Q264" t="inlineStr">
         <is>
           <t>https://www.fia.com/system/files/decision-document/2026_singapore_grand_prix_-_decision_-_car_44_-_alleged_leaving_the_track_and_gaining_an_advantage.pdf</t>
         </is>

</xml_diff>

<commit_message>
Add FIA document links for 2026 China, Canada, Great Britain, Netherlands and Hungary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -65863,6 +65863,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_23_-_breach_of_practice_start_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -65916,6 +65921,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_decision_-_car_12_-_alleged_impeding_of_car_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -65969,6 +65979,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_decision_-_car_10_-_alleged_impeding_of_car_3.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -66017,6 +66032,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_23_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -66068,6 +66088,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_12_-_causing_a_collision_with_car_6.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -66119,6 +66144,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_11_-_safety_car_ecu_minimum_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -66162,6 +66192,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_6_-_failing_to_follow_race_directors_instruction.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -66213,6 +66248,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_10_-_released_in_an_unsafe_condition.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -66261,6 +66301,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_23_-_changes_made_during_parc_ferme_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -66312,6 +66357,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_chinese_grand_prix_-_infringement_-_car_31_-_causing_a_collision_with_car_43.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -67396,6 +67446,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_16_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -67444,6 +67499,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_31_-_leaving_the_pitlane_after_the_end_of_the_session.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -67500,6 +67560,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_30_-_breach_of_article_c9.3.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -67548,6 +67613,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -67596,6 +67666,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_12_-_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -67644,6 +67719,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_77_-_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -67692,6 +67772,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_87_-_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -67740,6 +67825,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_10_-_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -67788,6 +67878,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_23_-_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -67836,6 +67931,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_18_-_starting_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -67887,6 +67987,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_27_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -67938,6 +68043,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_11_-_forcing_car_30_off_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -67986,6 +68096,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_decision_-_car_44_-_alleged_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -68039,6 +68154,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_decision_-_car_31_-_alleged_procedural_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -68095,6 +68215,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_14_-_unsafe_release_from_garage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -68242,6 +68367,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_decision_-_car_44_-_alleged_impeding_of_car_10.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -68290,6 +68420,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_decision_-_car_18_-_allegedly_impeded_car_27.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -68338,6 +68473,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_18_-_pu_elements_changed_under_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -68384,6 +68524,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_27_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -68430,6 +68575,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_77_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -68481,6 +68631,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_5_-_driving_unnecessarily_slowly_during_vsc.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -68529,6 +68684,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_27_-_starting_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -68580,6 +68740,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_81_-_collision_with_car_23.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -68623,6 +68788,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_decision_-_car_11_-_ignoring_blue_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -68676,6 +68846,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_30_-_starting_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -68727,6 +68902,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_63_-_unsafe_act.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -68770,6 +68950,11 @@
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_6_-_failing_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -71547,6 +71732,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_41_-_failing_to_follow_race_directors_instructions_sc2-sc1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -71595,6 +71785,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_30_-_abnormal_change_of_direction.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -71651,6 +71846,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_27_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -71699,6 +71899,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_23_-_failing_to_follow_race_directors_instructions_sc2-sc1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -71747,6 +71952,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_23_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -72109,6 +72319,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_infringement_-_car_11_-_causing_a_collision_with_car_14.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -72208,6 +72423,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Richard Norbury, Tanja Geilhausen, Pedro Lamy</t>
         </is>
       </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_british_grand_prix_-_decision_-_car_31_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -73025,6 +73245,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_11_-_starting_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -73501,6 +73726,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_87_-_ignoring_blue_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -73635,6 +73865,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_decision_-_car_10_-_alleged_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -73683,6 +73918,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_3_-_failure_to_follow_race_directors_instructions_reaching_the_grid.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -73736,6 +73976,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_5_-_red_light_at_pit_exit.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -73784,6 +74029,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_5_-_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -73832,6 +74082,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_11_-_changes_made_in_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -73880,6 +74135,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_14_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -73928,6 +74188,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_18_-_failure_to_follow_race_directors_instructions_reaching_the_grid.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -73976,6 +74241,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_22_-_failure_to_follow_race_directors_instructions_reaching_the_grid.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -74030,6 +74300,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_30_-_failure_to_follow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -74086,6 +74361,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_41_-_overtaking_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -74140,6 +74420,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_43_-_failure_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -74196,6 +74481,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_43_-_overtaking_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -74244,6 +74534,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_44_-_failure_to_follow_race_directors_instructions_reaching_the_grid.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -74292,6 +74587,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_55_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -74343,6 +74643,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_55_-_collision_with_car_23.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -74391,6 +74696,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_77_-_failure_to_follow_race_directors_instructions_reaching_the_grid.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -74444,6 +74754,11 @@
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
         </is>
       </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement_-_car_87_-_red_light_at_pit_exit.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -74485,6 +74800,11 @@
       <c r="P187" t="inlineStr">
         <is>
           <t>Felix Holter, Mathieu Rommerie, Tomas Kunac, Vitantonio Liuzzi, Stijn Drinkenburg</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_dutch_grand_prix_-_infringement-_car_55_-_driving_unnecessarily_slowly_during_sprint_qualifying.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FIA document links for 2026 Japan, Miami, Monaco, Hungary and Italy
Also correct Stroll's Canada unsafe release fine to 7500 and set two
Italy reconnaissance lap rows to Pre-Race.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -66415,6 +66415,11 @@
           <t>Gerd Ennser, Matthew Selley, Zhou Xiaoxu, Derek Warwick, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_japanese_grand_prix_-_decision_-_car_30_-_alleged_incident_with_car_55.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -66468,6 +66473,11 @@
           <t>Gerd Ennser, Matthew Selley, Zhou Xiaoxu, Derek Warwick, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_japanese_grand_prix_-_decision_-_car_23_-_alleged_incident_with_car_11.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -66516,6 +66526,11 @@
           <t>Gerd Ennser, Matthew Selley, Zhou Xiaoxu, Derek Warwick, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_japanese_grand_prix_-_decision_-_car_44_-_alleged_incident_with_car_3.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -66564,6 +66579,11 @@
           <t>Gerd Ennser, Matthew Selley, Zhou Xiaoxu, Derek Warwick, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_japanese_grand_prix_-_infringement_-_car_43_-_impeding_of_car_3.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -66612,6 +66632,11 @@
           <t>Gerd Ennser, Matthew Selley, Zhou Xiaoxu, Derek Warwick, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_japanese_grand_prix_-_infringement_-_car_81_-_impeding_of_car_27.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -66658,6 +66683,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_16_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -66709,6 +66739,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_23_-_track_limits.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -66810,6 +66845,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_41_-_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -66856,6 +66896,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_12_-_leaving_the_track_without_a_justifiable_reason_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -66909,6 +66954,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_5_-_technical_non-conformity_engine_intake_air_pressure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -66962,6 +67012,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_6_-_technical_nonconformity_floor_board.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -67005,6 +67060,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_77_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -67048,6 +67108,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_decision_-_car_31_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -67091,6 +67156,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_decision_-_car_23_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -67134,6 +67204,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_decision_-_car_14_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -67187,6 +67262,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_decision_-_car_3_-_alleged_incident_with_car_63.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -67240,6 +67320,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_decision_-_car_63_-_alleged_incident_with_car_3.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -67296,6 +67381,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_16_-_leaving_the_track_multiple_times_and_driving_in_an_unsafe_condition_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -67347,6 +67437,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_infringement_-_car_3_-_pit_exit_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -67400,6 +67495,11 @@
           <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_miami_grand_prix_-_decision_-_car_30_-_alleged_incident_with_car_10.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -68259,7 +68359,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>7000</v>
+        <v>7500</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -68269,6 +68369,11 @@
       <c r="P60" t="inlineStr">
         <is>
           <t>Garry Connelly, Tanja Geilhausen, Pedro Lamy, Marcel Demers</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_canadian_grand_prix_-_infringement_-_car_18_-_released_in_an_unsafe_condition.pdf</t>
         </is>
       </c>
     </row>
@@ -69011,6 +69116,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_1_-_media_commitment.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -69067,6 +69177,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_16_-_media_commitment.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -69113,6 +69228,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_63_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -69161,6 +69281,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_16_-_impeding_of_car_30.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -69209,6 +69334,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_41_-_impeding_of_car_81.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -69252,6 +69382,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_decision_-_car_30_-_alleged_leaving_the_pitlane_after_the_end_of_the_session.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -69298,6 +69433,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_14_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -69344,6 +69484,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_12_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -69400,6 +69545,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_1_-_technical_non-conformity_cds.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -69446,6 +69596,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_43_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -69492,6 +69647,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_23_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -69543,6 +69703,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_23_-_pit_lane_incident_with_car_41.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -69591,6 +69756,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_27_-_failure_to_follow_race_directors_instructions_-_tunnel.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -69639,6 +69809,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_11_-_false_start_-_out_of_position.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -69685,6 +69860,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_44_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -69731,6 +69911,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_63_-_pit_lane_speeding_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -69777,6 +69962,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_43_-_pit_lane_speeding_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -69823,6 +70013,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_10_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -69869,6 +70064,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_81_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -69917,6 +70117,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_10_-_pit_lane_speeding_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -69963,6 +70168,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_18_-_exceeded_track_limits.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -70014,6 +70224,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_11_-_false_start_-_out_of_position_at_restart.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -70062,6 +70277,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_decision_-_alleged_red_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -70110,6 +70330,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_decision_-_car_6_-_alleged_safety_car_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -70158,6 +70383,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_decision_-_car_44_-_alleged_safety_car_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -70262,6 +70492,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_infringement_-_car_27_-_causing_a_collision_with_car_55.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -70310,6 +70545,11 @@
           <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_monaco_grand_prix_-_decision_-_car_43_-_allegedly_causing_a_collision_with_car_55.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -73298,6 +73538,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_11_-_changes_made_under_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -73344,6 +73589,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_6_-_pit_lane_speeding_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -73392,6 +73642,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_55_-_erratic_driving_in_turn_12_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -73435,6 +73690,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_12_-_alleged_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -73484,6 +73744,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_12_-_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -73535,6 +73800,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_44_-_unnecessarily_impeding_of_car_81.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -73581,6 +73851,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_44_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -73629,6 +73904,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_decision_-_car_55_-_alleged_erratic_driving_in_turn_9.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -73680,6 +73960,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_infringement_-_car_55_-_collision_with_car_81.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -73774,6 +74059,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_decision_-_car_16_-_alleged_failure_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -73817,6 +74107,11 @@
           <t>Garry Connelly, Matthew Selley, Richa Mergulhao, Vitantonio Liuzzi, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_hungarian_grand_prix_-_decision_-_car_3_-_alleged_erratic_driving_in_turn_12.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -74860,6 +75155,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_23_-_failure_to_slow_for_double_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -74916,6 +75216,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_25_-_technical_non-conformity_cds.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -74964,6 +75269,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_30_-_changes_made_under_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -75010,6 +75320,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_30_-_change_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -75053,6 +75368,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_decision_-_car_22_-_alleged_start_procedure_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -75101,6 +75421,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_decision_-_car_30_-_turn_4_incident_with_car_27.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -75149,6 +75474,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_decision_-_car_63_-_alleged_failure_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -75174,7 +75504,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Pre-Race</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -75195,6 +75525,11 @@
       <c r="P195" t="inlineStr">
         <is>
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_11_-_failure_to_follow_race_directors_instruction_-_pit_exit.pdf</t>
         </is>
       </c>
     </row>
@@ -75243,6 +75578,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_11_-_failure_to_follow_race_directors_instruction_-_turns_1_and_2.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -75289,6 +75629,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_12_-_changes_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -75335,6 +75680,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_12_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -75383,6 +75733,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_14_-_pu_elements_changed_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -75431,6 +75786,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_18_-_impeding_of_car_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -75477,6 +75837,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_23_-_changes_to_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -75520,6 +75885,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_23_-_failure_to_follow_race_directors_instructions_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -75545,7 +75915,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Pre-Race</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -75566,6 +75936,11 @@
       <c r="P203" t="inlineStr">
         <is>
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_43_-_failure_to_follow_race_directors_instruction_-_practice_start.pdf</t>
         </is>
       </c>
     </row>
@@ -75616,6 +75991,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
         </is>
       </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_55_-_failure_to_slow_for_double_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -75665,6 +76045,11 @@
       <c r="P205" t="inlineStr">
         <is>
           <t>Garry Connelly, Mathieu Remmerie, Vitantonio Liuzzi, Iacopo Arcangeli</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_italian_grand_prix_-_infringement_-_car_81_-_impeding_of_car_30.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 2026 United States GP stewards decisions (Round 18)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -65049,7 +65049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q264"/>
+  <dimension ref="A1:Q276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="32.21875" customWidth="1" min="7" max="7"/>
@@ -79385,6 +79385,670 @@
         </is>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B265" t="n">
+        <v>18</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Franco Colapinto</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Alpine</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>FP1</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>New power unit element(s)</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M265" t="n">
+        <v>10</v>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_43_-_pu_element.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B266" t="n">
+        <v>18</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>FP1</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>New power unit element(s)</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M266" t="n">
+        <v>20</v>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q266" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_5_-_pu_elements.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B267" t="n">
+        <v>18</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Arvid Lindblad</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>FP1</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>New power unit element(s)</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M267" t="n">
+        <v>5</v>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_41_-_changes_to_pu_element_corrected.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B268" t="n">
+        <v>18</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>George Russell</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>FP2</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Forcing another car off the track</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Charles Leclerc</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>Both cars on preparation laps</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q268" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_decision_-_car_63_-_alleged_forcing_another_driver_off_the_track.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B269" t="n">
+        <v>18</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>FP3</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>New power unit element(s)</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M269" t="n">
+        <v>60</v>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_5_-_additional_changes_to_pu_elements.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B270" t="n">
+        <v>18</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Nico Hulkenberg</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>FP3</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Pit Lane Incident</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>Pulled out in front of another car while performing a practice start</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_27_-_alleged_pit_lane_incident.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B271" t="n">
+        <v>18</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Isack Hadjar</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>FP3</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Driving Erratically</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Swerved towards another car after aborting a lap</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Alexander Albon</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_6_-_driving_erratically.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B272" t="n">
+        <v>18</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>FP3</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Impeding</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Lewis Hamilton</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_5_-_impeding_of_car_44.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B273" t="n">
+        <v>18</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Lance Stroll</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Aston Martin</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Changes made under parc ferme</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>New PU elements fitted, suspension setup changed and work beyond covers-off time under parc ferme</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Pit Lane</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_18_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B274" t="n">
+        <v>18</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Leaving the Track and Gaining an Advantage</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Franco Colapinto</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>No Further Action</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>Stewards could not determine which car was ahead at the apex</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_decision_-_car_5_-_alleged_leaving_the_track_and_gaining_and_advantage.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B275" t="n">
+        <v>18</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Oliver Bearman</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Haas</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Causing a Collision</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Pierre Gasly</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Time Penalty</t>
+        </is>
+      </c>
+      <c r="K275" t="n">
+        <v>10</v>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_87_-_causing_a_collision.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B276" t="n">
+        <v>18</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>George Russell</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Mercedes</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Leaving the Track and Gaining an Advantage</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Oscar Piastri</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Time Penalty</t>
+        </is>
+      </c>
+      <c r="K276" t="n">
+        <v>5</v>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>Standard 10 second penalty reduced to 5 seconds as a first lap incident</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Matthew Selley, Pedro Lamy, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_united_states_grand_prix_-_infringement_-_car_63_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add FIA document links for 2025 (157 rows) and fix China practice start sessions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -52133,6 +52133,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_23_-_unsafe_release_from_garage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -52184,6 +52189,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_23_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -52240,6 +52250,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_14_-_fan_engagement_activity.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -52296,6 +52311,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_12_-_unsafe_release_from_garage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -52352,6 +52372,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_18_-_fan_engagement_activity.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -52411,6 +52436,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_18_-_more_than_one_change_of_direction.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -52464,6 +52494,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_decision_-_car_4_-_alleged_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -52523,6 +52558,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_30_-_erratic_driving.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -52581,6 +52621,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_decision_-_car_27_-_alleged_causing_a_collision_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -52640,6 +52685,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_87_-_more_than_one_change_of_direction.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -52698,6 +52748,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_decision_-_car_10_-_alleged_causing_a_collision_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -52749,6 +52804,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_10_-_leaving_the_track_without_a_justifiable_reason_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -52805,6 +52865,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_22_-_impeding_of_car_4_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -52864,6 +52929,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Derek Warwick, Mohammed Al Hashmi</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_abu_dhabi_grand_prix_-_infringement_-_car_22_-_more_than_one_change_of_direction.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -52912,6 +52982,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_decision_-_car_23_-_failing_to_maintain_distance_behind_the_safety_car_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -52960,6 +53035,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_decision_-_car_14_-_failing_to_maintain_distance_behind_the_safety_car.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -53016,6 +53096,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_infringement_-_car_5_-_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -53077,6 +53162,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_infringement_-_car_12_-_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -53125,6 +53215,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_decision_-_car_44_-_failing_to_maintain_distance_behind_the_safety_car.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -53178,6 +53273,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_infringement_-_car_30_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -53231,6 +53331,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_infringement_-_car_87_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -53279,6 +53384,11 @@
           <t>Garry Connelly, Gerd Ennser, Tanja Geilhausen, Matthew Selley</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_australian_grand_prix_-_decision_-_car_22_-_failing_to_maintain_distance_behind_the_safety_car.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -53332,6 +53442,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_decision_-_car_43_-_alleged_forcing_another_driver_off_of_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -53391,6 +53506,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_infringement_-_car_43_-_forcing_car_81_off_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -53439,6 +53559,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_infringement_-_car_63_-_pit_lane_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -53490,6 +53615,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_infringement_-_car_12_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -53554,6 +53684,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_infringement_-_car_12_-_causing_a_collision_with_car_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -53607,6 +53742,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_infringement_-_car_44_-_impeding_of_car_12.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -53666,6 +53806,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_infringement_-_car_22_-_causing_a_collision_with_car_43_in_turn_4.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -53719,6 +53864,11 @@
           <t>Felix Holter, Garry Connelly, Derek Warwick, Wilhelm Singer</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_austrian_grand_prix_-_decision_-_car_22_-_alleged_forcing_car_18_off_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -53778,6 +53928,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Enrique Bernoldi, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_azerbaijan_grand_prix_-_infringement_-_car_23_-_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -53831,6 +53986,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Enrique Bernoldi, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_azerbaijan_grand_prix_-_infringement_-_car_31_-_failure_of_rear_wing_main_plane_tip_deflection_test.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -53882,6 +54042,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Enrique Bernoldi, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_azerbaijan_grand_prix_-_infringement_-_car_14_false_start_-_moving_before_signal.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -53930,6 +54095,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Enrique Bernoldi, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_azerbaijan_grand_prix_-_infringement_-_car_12_-_failure_to_slow_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -53983,6 +54153,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Enrique Bernoldi, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_azerbaijan_grand_prix_-_infringement_-_car_27_-_failure_to_slow_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -54031,6 +54206,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Enrique Bernoldi, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_azerbaijan_grand_prix_-_infringement_-_car_81_-_failure_to_slow_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -54082,6 +54262,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Enrique Bernoldi, Danil Solomin</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_azerbaijan_grand_prix_-_infringement_-_car_81_false_start_-_moving_before_signal.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -54138,6 +54323,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_23_-_impeding_of_car_46.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -54197,6 +54387,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_55_-_forcing_another_driver_off_the_track_corrected.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -54248,6 +54443,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_63_-_alleged_failure_to_follow_race_directors_instructions_fast_lane.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -54301,6 +54501,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_63_-_alleged_drs_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -54352,6 +54557,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_7_-_leaving_the_track_without_a_justifiable_reason_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -54403,6 +54613,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_12_-_alleged_failure_to_follow_race_directors_instructions_fast_lane.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -54454,6 +54669,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_4_-_incorrect_starting_position.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -54513,6 +54733,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_30_-_causing_a_collision_with_car_18_at_t2.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -54572,6 +54797,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_30_-_causing_a_collision_with_car_27_at_t1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -54620,6 +54850,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_27_-_track_limits.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -54673,6 +54908,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_27_-_technical_non-compliance_plank_assembly.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -54726,6 +54966,11 @@
           <t>Garry Connelly, Matheiu Remmerie, Vitantonio Liuzzi, Mazen Al Hilli</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_bahrain_grand_prix_-_infringement_-_car_22_-_pit_lane_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -54779,6 +55024,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_infringement_-_car_55_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -54832,6 +55082,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_infringement_-_car_14_-_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -54885,6 +55140,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_infringement_-_car_43_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -54933,6 +55193,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_decision_-_car_63_-_driving_unnecessarily_slowly.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -54986,6 +55251,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_infringement_-_car_12_-_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -55039,6 +55309,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_infringement_-_car_44_-_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -55092,6 +55367,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_infringement_-_car_27_-_pit_lane_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -55145,6 +55425,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_decision_-_car_10_-_allegedly_impeding_car_22.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -55193,6 +55478,11 @@
           <t>Garry Connelly, Felix Holter, Vitantonio Liuzzi, Loic Bacquelaine</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_belgian_grand_prix_-_infringement_-_car_22_-_driving_unnecessarily_slow.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -55795,6 +56085,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_23_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -55843,6 +56138,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_55_-_safety_car_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -55891,6 +56191,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_16_-_safety_car_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -55939,6 +56244,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_31_-_failure_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -55992,6 +56302,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_31_-_alleged_erratic_driving_corrected.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -56040,6 +56355,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_31_-_safety_car_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -56098,6 +56418,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_decision_-_car_5_-_alleged_red_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -56146,6 +56471,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_63_-_failed_to_follow_race_director_instruction.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -56197,6 +56527,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_63_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -56253,6 +56588,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_63_-_pit_lane_speeding_2nd.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -56309,6 +56649,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_6_-_impeding_car_55.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -56357,6 +56702,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_12_-_safety_car_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -56416,6 +56766,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_18_-_forcing_another_driver_off_of_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -56472,6 +56827,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_4_-_collision_with_car_81.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -56525,6 +56885,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_30_-_pu_elements_and_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -56578,6 +56943,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_87_-_failure_to_follow_race_directors_instructions_corrected.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -56629,6 +56999,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_81_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -56677,6 +57052,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_81_-_safety_car_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -56730,6 +57110,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_10_-_pu_elements.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -56778,6 +57163,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_10_-_safety_car_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -56837,6 +57227,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Derek Warwick, Marcel Demers</t>
         </is>
       </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_canadian_grand_prix_-_infringement_-_car_22_-_overtaking_under_red_flag_conditions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -56885,6 +57280,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_decision_-_car_16_-_alleged_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -56938,6 +57338,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_16_-_technical_non-compliance_weight.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -56963,7 +57368,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Pre-Race</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -56989,6 +57394,11 @@
       <c r="P94" t="inlineStr">
         <is>
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_5_-_practice_start.pdf</t>
         </is>
       </c>
     </row>
@@ -57047,6 +57457,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_6_-_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -57106,6 +57521,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_7_-_incident_with_car_5.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -57165,6 +57585,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_7_-_forcing_another_driver_off_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -57213,6 +57638,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_decision_-_car_18_-_alleged_failure_to_follow_race_directors_instructions_sc2-sc1_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -57266,6 +57696,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_44_-_technical_non-compliance_plank_assembly.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -57324,6 +57759,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_decision_-_car_30_-_alleged_incident_with_car_7.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -57377,6 +57817,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_30_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -57430,6 +57875,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_27_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -57455,7 +57905,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Pre-Race</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -57481,6 +57931,11 @@
       <c r="P103" t="inlineStr">
         <is>
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_27_-_practice_start.pdf</t>
         </is>
       </c>
     </row>
@@ -57536,6 +57991,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_decision_-_car_87_-_alleged_impeding_of_car_18.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -57589,6 +58049,11 @@
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
         </is>
       </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_10_-_technical_non-compliance_weight.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -57614,7 +58079,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Pre-Race</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -57640,6 +58105,11 @@
       <c r="P106" t="inlineStr">
         <is>
           <t>Nish Shetty, Gerd Ennser, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_chinese_grand_prix_-_infringement_-_car_22_-_practice_start.pdf</t>
         </is>
       </c>
     </row>
@@ -57695,6 +58165,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_infringement_-_car_55_-_dangerous_driving.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -57753,6 +58228,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_decision_-_car_31_-_incident_with_car_87.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -57806,6 +58286,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_infringement_-_car_43_-_pu_elements_corrected.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -57864,6 +58349,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_decision_-_car_6_-_alleged_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -57918,6 +58408,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_infringement_-_car_87_-_failure_to_comply_with_red_flag_corrected.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -57976,6 +58471,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_decision_-_car_87_-_incident_with_car_31.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -58030,6 +58530,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_infringement_-_car_81_-_safety_car_procedure.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -58089,6 +58594,11 @@
           <t>Nish Shetty, Mathieu Remmerie, Vitantonio Liuzzi, Richard Norbury</t>
         </is>
       </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_british_grand_prix_-_infringement_-_car_22_-_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -58148,6 +58658,11 @@
           <t>Felix Holter, Matthew Selley, Derek Warwick, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_hungarian_grand_prix_-_infringement_-_car_16_-_erratic_driving.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -58196,6 +58711,11 @@
           <t>Felix Holter, Matthew Selley, Derek Warwick, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_hungarian_grand_prix_-_decision_-_car_1_-_alleged_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -58254,6 +58774,11 @@
           <t>Felix Holter, Matthew Selley, Derek Warwick, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_hungarian_grand_prix_-_decision_-_car_1_-_alleged_forcing_another_driver_off_of_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -58305,6 +58830,11 @@
           <t>Felix Holter, Matthew Selley, Derek Warwick, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_hungarian_grand_prix_-_infringement_-_car_27_-_false_start.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -58364,6 +58894,11 @@
           <t>Felix Holter, Matthew Selley, Derek Warwick, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_hungarian_grand_prix_-_infringement_-_car_10_-_colliding_with_car_55.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -58417,6 +58952,11 @@
           <t>Felix Holter, Matthew Selley, Derek Warwick, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_hungarian_grand_prix_-_infringement_-_car_22_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -58475,6 +59015,11 @@
           <t>Felix Holter, Matthew Selley, Derek Warwick, Istvan Moni</t>
         </is>
       </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_hungarian_grand_prix_-_decision_-_car_22_-_alleged_forcing_another_driver_off_of_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -58526,6 +59071,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Valerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_emilia_romagna_grand_prix_-_infringement_-_car_55_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -58577,6 +59127,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Valerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_emilia_romagna_grand_prix_-_infringement_-_car_16_-_tyre_operating_procedures.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -58635,6 +59190,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Valerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_emilia_romagna_grand_prix_-_decision_-_car_16_-_alleged_forcing_another_driver_off_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -58686,6 +59246,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Valerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_emilia_romagna_grand_prix_-_infringement_-_car_43_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -58737,6 +59302,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Valerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_emilia_romagna_grand_prix_-_infringement_-_car_43_-_alleged_failure_to_follow_race_directors_instructions_fast_lane.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -58790,6 +59360,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Valerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_emilia_romagna_grand_prix_-_decision_-_car_5_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -58843,6 +59418,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Valerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_emilia_romagna_grand_prix_-_infringement_-_car_22_-_pu_elements_and_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -58891,6 +59471,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_55_-_failure_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -58950,6 +59535,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_31_-_forcing_another_driver_off_the_track.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -58998,6 +59588,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_14_-_failing_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -59051,6 +59646,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_decision_-_car_5_overtook_car_30_in_a_yellow_flag_zone.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -59099,6 +59699,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_6_-_failing_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -59152,6 +59757,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_6_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -59211,6 +59821,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_12_-_erratic_driving_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -59259,6 +59874,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_18_-_failing_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -59318,6 +59938,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_87_-_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -59366,6 +59991,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_decision_-_car_81_-_failure_to_follow_race_directors_instructions_-_fast_lane.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -59419,6 +60049,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Velerio Brizzolari</t>
         </is>
       </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_italian_grand_prix_-_infringement_-_car_10_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -59465,6 +60100,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_55_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -59516,6 +60156,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_55_-_impeding_of_car_44.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -59567,6 +60212,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_55_-_late_attendance_of_national_anthem.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -59613,6 +60263,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_12_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -59656,6 +60311,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_18_-_failure_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -59699,6 +60359,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_44_-_failure_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -59742,6 +60407,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_1_-_failure_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -59785,6 +60455,11 @@
           <t>Garry Connelly, Mathieu Remmerie, Pedro Lamy, Kazuhiro Tsuge</t>
         </is>
       </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_japanese_grand_prix_-_infringement_-_car_81_-_failure_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -59839,6 +60514,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_23_-_collision_with_car_44_in_turn_14.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -59887,6 +60567,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_23_-_exceeded_speed_limit_when_leaving_the_grid.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -59940,6 +60625,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_decision_-_car_55_-_alleged_rejoining_the_track_unsafely.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -60034,6 +60724,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_43_-_electronic_return_of_tyres.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -60131,6 +60826,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_5_-_causing_a_collision_with_car_18_in_turn_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -60179,6 +60879,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_decision_-_car_63_-_alleged_failure_to_submit_setup_sheet.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -60227,6 +60932,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_decision_-_car_12_-_alleged_failure_to_submit_setup_sheet.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -60273,6 +60983,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_12_-_moved_prior_to_start_signal.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -60321,6 +61036,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_4_-_technical_non-conformity_plank_assembly.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -60420,6 +61140,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_decision_-_car_30_-_turn_1_incident_with_car_81.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -60468,6 +61193,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_81_-_technical_non-conformity_plank_assembly_corrected.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -60516,6 +61246,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_22_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -62137,6 +62872,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_decision_-_williams_petition_for_right_of_review_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -62195,6 +62935,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_decision_-_car_16_-_alleged_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -62243,6 +62988,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_decision_-_car_5_alleged_driving_under_unsafe_conditions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -62299,6 +63049,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_infringement_-_car_63_-_pit_lane_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -62357,6 +63112,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_decision_-_car_63_-_alleged_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -62408,6 +63168,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_decision_-_car_12_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -62467,6 +63232,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_infringement_-_car_12_-_causing_a_collision_with_car_16.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -62521,6 +63291,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_infringement_-_car_44_-_failing_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -62574,6 +63349,11 @@
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
         </is>
       </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_infringement_-_car_87_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -62628,6 +63408,11 @@
       <c r="P204" t="inlineStr">
         <is>
           <t>Nish Shetty, Matthew Selley, Pedro Lamy, Natalie Corsmit</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_dutch_grand_prix_-_infringement_-_car_81_-_pit_lane_incident.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FIA document links for 75 more 2025 rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -55531,6 +55531,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_55_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -55579,6 +55584,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_31_-_pu_elements_and_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -55622,6 +55632,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_44_-_failing_to_slow_for_double_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -55676,6 +55691,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_44_-_causing_a_collision_with_car_43_in_turn_15.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -55730,6 +55750,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_corrected_-_sprint_infringement_-_car_30_-_causing_a_collision_with_car_87_at_t4.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -55778,6 +55803,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_1_-_pu_elements_and_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -55832,6 +55862,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_87_-_driving_in_a_manner_deemed_potentially_dangerous.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -55886,6 +55921,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_corrected_race_-_infringement_-_car_81_-_causing_a_collision_with_car_12_in_turn_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -55934,6 +55974,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_22_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -55988,6 +56033,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_22_-_causing_a_collision_with_car_18_in_turn_8.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -56034,6 +56084,11 @@
           <t>Gerd Ennser, Mathieu Remmerie, Tanja Geilhausen, Pedro Lamy, Luciano Burti</t>
         </is>
       </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_sao_paulo_grand_prix_-_infringement_-_car_22_-_failure_to_serve_a_time_penalty_during_a_pit_stop.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -60678,6 +60733,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_decision_-_car_16_-_alleged_failure_to_leave_the_gar_in_gear_and_turn_off_ers.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -60772,6 +60832,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_decision_-_car_5_-_alleged_failure_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -61087,6 +61152,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Vitantonio Liuzzi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_las_vegas_grand_prix_-_infringement_-_car_44_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -61299,6 +61369,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Pedro Lamy, Alfonso Oros Trigueros</t>
         </is>
       </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_mexico_city_grand_prix_-_infringement_-_car_36_-_impeding_car_89_in_turn_9.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -61345,6 +61420,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Pedro Lamy, Alfonso Oros Trigueros</t>
         </is>
       </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_mexico_city_grand_prix_-_infringement_-_car_55_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -61393,6 +61473,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Pedro Lamy, Alfonso Oros Trigueros</t>
         </is>
       </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_mexico_city_grand_prix_-_infringement_-_car_55_-_pit_lane_speeding_2nd.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -61444,6 +61529,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Pedro Lamy, Alfonso Oros Trigueros</t>
         </is>
       </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_mexico_city_grand_prix_-_infringement_-_car_44_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -61487,6 +61577,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Pedro Lamy, Alfonso Oros Trigueros</t>
         </is>
       </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_mexico_city_grand_prix_-_decision_-_car_44_-_alleged_failing_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -61540,6 +61635,11 @@
           <t>Gerd Ennser, Matthew Selley, Natalie Corsmit, Pedro Lamy, Alfonso Oros Trigueros</t>
         </is>
       </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_mexico_city_grand_prix_-_decision_-_car_44_-_alleged_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -61586,6 +61686,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_23_-_safety_car_ecu_minimum_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -61629,6 +61734,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_23_-_pit_lane_incident.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -61682,6 +61792,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_decision_-_car_55_-_alleged_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -61725,6 +61840,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_55_-_failing_to_slow_for_yellow_flag.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -61773,6 +61893,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_16_-_driving_a_car_in_an_unsafe_condition.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -61824,6 +61949,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_31_-_impeding_car_4.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -61870,6 +62000,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_7_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -61913,6 +62048,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_4_-_unsafe_condition.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -61966,6 +62106,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_decision_-_car_44_-_alleged_causing_a_collision.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -62020,6 +62165,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_30_-_collision_with_car_14.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -62071,6 +62221,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_1_-_unsafe_release_from_a_pit_stop.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -62122,6 +62277,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_87_-_unsafe_release_from_a_pit_stop.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -62170,6 +62330,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_10_-_corrected_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -62213,6 +62378,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_10_-_failing_to_slow_for_yellow_flag.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -62261,6 +62431,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_22_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -62307,6 +62482,11 @@
           <t>Felix Holter, Mathieu Remmerie, Derek Warwick, Steve Pence</t>
         </is>
       </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_miami_grand_prix_-_infringement_-_car_22_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -62355,6 +62535,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_decision_-_car_55_-_alleged_failure_to_comply_with_red_flag_in_p2.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -62403,6 +62588,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_decision_-_car_43_-_alleged_failure_to_comply_with_red_flag.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -62451,6 +62641,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_infringement_-_car_63_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -62505,6 +62700,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_infringement_-_car_18_-_incident_with_car_16_in_turn_6.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -62556,6 +62756,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_infringement_-_car_18_-_impeding_car_10_in_turn_10.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -62607,6 +62812,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_infringement_-_car_44_-_impeding_of_car_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -62661,6 +62871,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_infringement_-_car_87_-_alleged_failure_to_comply_with_red_flag.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -62712,6 +62927,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_infringement_-_haas_-_unsafe_condition_of_car_87.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -62760,6 +62980,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_infringement_-_car_10_-_incident_with_car_22.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -62808,6 +63033,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Vitantonio Liuzzi, Jean-Francois Calmes</t>
         </is>
       </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_monaco_grand_prix_-_decision_-_car_22_-_alleged_failing_to_slow_for_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -63463,6 +63693,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_decision_-_car_23_-_alleged_pit_lane_incident_with_car_31.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -63509,6 +63744,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_55_-_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -63555,6 +63795,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_31_-_false_start_-_moving_before_signal.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -63603,6 +63848,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_43_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -63651,6 +63901,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_43_-_changes_made_during_parc_ferme_0.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -63694,6 +63949,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_decision_-_car_6_-_alleged_driving_in_an_unsafe_condition.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -63740,6 +64000,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_12_-_leaving_the_track_without_a_justifiable_reason_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -63788,6 +64053,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_18_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -63834,6 +64104,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_18_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -63882,6 +64157,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_44_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -63925,6 +64205,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_27_-_failure_to_follow_race_directors_instructions.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -63978,6 +64263,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_decision_-_car_27_-_alleged_causing_a_collision_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -64021,6 +64311,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_87_-_released_in_an_unsafe_condition.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -64069,6 +64364,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_10_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -64115,6 +64415,11 @@
           <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Amro Al Hamad</t>
         </is>
       </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_qatar_grand_prix_-_infringement_-_car_22_-_leaving_the_track_without_a_justifiable_reason_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -64158,6 +64463,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_infringement_-_car_7_-_failure_to_follow_race_directors_instructions_pit_entry_-_1st_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -64206,6 +64516,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_infringement_-_car_7_-_failure_to_follow_race_directors_instructions_pit_entry_-_2nd_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -64254,6 +64569,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_decision_-_car_44_-_alleged_impeding_of_car_23.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -64297,6 +64617,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_infringement_-_car_30_-_failure_to_follow_race_directors_instructions_pit_entry_-_1st_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -64345,6 +64670,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_infringement_-_car_30_-_failure_to_follow_race_directors_instructions_pit_entry_-_2nd_time.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -64396,6 +64726,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_infringement_-_car_30_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -64452,6 +64787,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_infringement_-_car_1_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -64505,6 +64845,11 @@
           <t>Nish Shetty, Loic Bacquelaine, Enrique Bernoldi, Hasan Al Aldabi</t>
         </is>
       </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_saudi_arabian_grand_prix_-_decision_-_car_22_-_alleged_causing_a_collision_with_car_10_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -64553,6 +64898,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_infringement_-_car_23_-_technical_regulations_drs.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -64601,6 +64951,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_infringement_-_car_23_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -64649,6 +65004,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_infringement_-_car_23_-_use_of_pit_exit_lane_during_reconnaissance_lap.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -64697,6 +65057,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_infringement_-_car_55_-_technical_regulations_drs.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -64923,6 +65288,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_infringement_-_car_44_-_leaving_the_track_without_a_justifiable_reason_multiple_times.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -65012,6 +65382,11 @@
       <c r="P238" t="inlineStr">
         <is>
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
+        </is>
+      </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_infringement_-_car_10_-_changes_made_during_parc_ferme.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FIA document links for the final 21 rows of 2025
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -65113,6 +65113,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_infringement_-_car_16_-_unsafe_release.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -65156,6 +65161,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_decision_-_car_5_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -65199,6 +65209,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_decision_-_car_63_-_allegedly_failing_to_slow_under_yellow_flags.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -65242,6 +65257,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_decision_-_car_44_-_allegedly_failing_to_comply_with_a_red_flag.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -65336,6 +65356,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_decision_-_car_27_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -65432,6 +65457,11 @@
           <t>Gerd Ennser, Loic Bacquelaine, Natalie Corsmit, Derek Warwick, Paul Ng</t>
         </is>
       </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_singapore_grand_prix_-_decision_-_car_22_-_alleged_yellow_flag_infringement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -65483,6 +65513,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_infringement_-_car_23_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -65536,6 +65571,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_decision_-_car_16_-_alleged_collision_with_car_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -65579,6 +65619,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_decision_-_car_43_-_allegedly_leaving_the_pit_lane_with_a_technical_issue.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -65627,6 +65672,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_infringement_-_car_18_-_post-qualifying_weighing.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -65680,6 +65730,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_decision_-_car_30_-_alleged_collision_with_car_23.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -65733,6 +65788,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_decision_-_car_30_-_alleged_collision_with_car_87.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -65786,6 +65846,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_decision_-_car_1_-_alleged_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -65840,6 +65905,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_infringement_-_car_1_-_causing_a_collision_with_car_63_at_t5.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -65893,6 +65963,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_decision_-_car_1_-_alleged_collision_with_car_16.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -65944,6 +66019,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_infringement_-_car_87_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -65992,6 +66072,11 @@
           <t>Nish Shetty, Matthew Selley, Vitantonio Liuzzi, David Domingo</t>
         </is>
       </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_spanish_grand_prix_-_infringement_-_car_22_-_changes_made_during_parc_ferme.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -66046,6 +66131,11 @@
           <t>Felix Holter, Mathew Selley, Enrique Bernoldi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_united_states_grand_prix_-_infringement_-_car_55_-_causing_a_collision_with_car_12_in_turn_15.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -66092,6 +66182,11 @@
           <t>Felix Holter, Mathew Selley, Enrique Bernoldi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_united_states_grand_prix_-_infringement_-_car_5_-_pit_lane_speeding.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -66146,6 +66241,11 @@
           <t>Felix Holter, Mathew Selley, Enrique Bernoldi, Steve Pence</t>
         </is>
       </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_united_states_grand_prix_-_infringement_-_car_18_-_causing_a_collision_with_car_31.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -66195,6 +66295,11 @@
       <c r="P254" t="inlineStr">
         <is>
           <t>Felix Holter, Mathew Selley, Enrique Bernoldi, Steve Pence</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2025_united_states_grand_prix_-_infringement_-_car_87_-_leaving_the_track_and_gaining_an_advantage.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 2026 Mexico City GP stewards decisions so far (Round 19)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -66314,7 +66314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q276"/>
+  <dimension ref="A1:Q281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="32.21875" customWidth="1" min="7" max="7"/>
@@ -81314,6 +81314,307 @@
         </is>
       </c>
     </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B277" t="n">
+        <v>19</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Valtteri Bottas</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Cadillac</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>FP1</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>New power unit element(s)</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Grid Penalty</t>
+        </is>
+      </c>
+      <c r="M277" t="n">
+        <v>50</v>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Omar Chavez Jimenez</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_mexico_city_grand_prix_-_infringement_-_car_77_-_pu_elements.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B278" t="n">
+        <v>19</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Freddie Slater</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>FP1</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Unsafe Release</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Fine</t>
+        </is>
+      </c>
+      <c r="L278" t="n">
+        <v>7500</v>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>Released with a cooling fan still attached to the radiator intake</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Omar Chavez Jimenez</t>
+        </is>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_mexico_city_grand_prix_-_infringement_-_car_98_-_released_in_an_unsafe_condition.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B279" t="n">
+        <v>19</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Gabriel Bortoleto</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Audi</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>FP2</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Technical Infringement</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Covered the floor and obstructed the view of the car while mechanics worked on it</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Fine</t>
+        </is>
+      </c>
+      <c r="L279" t="n">
+        <v>5000</v>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Omar Chavez Jimenez</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_mexico_city_grand_prix_-_infringement_-_car_5_-_covering_components.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B280" t="n">
+        <v>19</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Max Verstappen</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Red Bull</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>FP2</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Dangerous Driving</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Series of moves with Car 30 from Turn 12 to Turn 14</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Liam Lawson</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Grid Penalty, Penalty Points</t>
+        </is>
+      </c>
+      <c r="M280" t="n">
+        <v>1</v>
+      </c>
+      <c r="N280" t="n">
+        <v>1</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>Stewards escalated from a warning to a grid penalty after a warning at the Team Managers meeting about Free Practice incidents</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Omar Chavez Jimenez</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_mexico_city_grand_prix_-_infringement_-_car_3_-_turn_14_incident_with_car_30_.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B281" t="n">
+        <v>19</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Liam Lawson</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Racing Bulls</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>FP2</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Dangerous Driving</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Series of moves with Car 3 from Turn 12 to Turn 14</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Max Verstappen</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Grid Penalty, Penalty Points</t>
+        </is>
+      </c>
+      <c r="M281" t="n">
+        <v>1</v>
+      </c>
+      <c r="N281" t="n">
+        <v>1</v>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>Stewards escalated from a warning to a grid penalty after a warning at the Team Managers meeting about Free Practice incidents</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>Garry Connelly, Loic Bacquelaine, Derek Warwick, Omar Chavez Jimenez</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>https://www.fia.com/system/files/decision-document/2026_mexico_city_grand_prix_-_infringement_-_car_30_-_turn_14_incident_with_car_3_.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>